<commit_message>
feat(inventario): plantilla con hojas Instrucciones/Sitios/Listas + generador
La plantilla de carga ahora incluye una hoja de Instrucciones (cómo llenar
xlsx/csv, reglas y diccionario de las 23 columnas), filas de ejemplo en la
hoja Sitios y una hoja Listas con los valores válidos. Se agrega el script
generador scripts/generar-plantilla-inventario.mjs para regenerarla.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/web/public/plantilla-sitios-set.xlsx
+++ b/apps/web/public/plantilla-sitios-set.xlsx
@@ -3,7 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sitios" sheetId="1" r:id="rId1"/>
+    <sheet name="Instrucciones" sheetId="1" r:id="rId1"/>
+    <sheet name="Sitios" sheetId="2" r:id="rId2"/>
+    <sheet name="Listas" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +399,460 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:D42"/>
+  <cols>
+    <col min="1" max="1" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="64.83203125" customWidth="1"/>
+    <col min="4" max="4" width="52.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>SPACES OS — Plantilla de carga de inventario (sitios / pantallas)</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Cómo usar esta plantilla:</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>1) Captura tus sitios en la hoja "Sitios" (una fila por sitio).</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>2) BORRA las 2 filas de EJEMPLO antes de importar.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>3) Guarda el archivo como .xlsx (o exporta la hoja "Sitios" como .csv) y súbelo en Inventario → Importar.</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Reglas importantes:</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>• Campos OBLIGATORIOS: nombre, exhibicion, unidad, tarifa_publicada, costo_compra. Si falta uno, la fila se rechaza.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>• exhibicion solo acepta: fijo o digital.</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>• Si exhibicion = fijo, la unidad SOLO puede ser "mensual" o "catorcenal" (cualquier otra rechaza la fila).</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>• Si dejas latitud/longitud vacías, el sitio se crea "pendiente de verificación" con coordenadas por default.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>• tarifa_publicada y costo_compra van SIN IVA, como número (sin $ ni comas). Ej: 85000.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>• Los valores de catálogo (tipo_medio, unidad, exhibicion, si/no) están en la hoja "Listas".</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>• No cambies los nombres de las columnas ni el nombre de la hoja "Sitios".</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>• ¿Usas CSV? Mismas columnas y mismo orden que la hoja "Sitios"; la primera fila debe ser el encabezado.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Diccionario de columnas:</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Columna</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Obligatorio</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Descripción</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Valores válidos / formato</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>codigo_proveedor</v>
+      </c>
+      <c r="B20" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Tu clave interna del sitio (la del proveedor).</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B21" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Nombre visible del sitio o pantalla.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>tipo_medio</v>
+      </c>
+      <c r="B22" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Tipo de soporte físico.</v>
+      </c>
+      <c r="D22" t="str">
+        <v>espectacular · muro · valla · parabus · mupi · publitienda · puente · otro</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>exhibicion</v>
+      </c>
+      <c r="B23" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C23" t="str">
+        <v>¿La pieza es impresa (fija) o pantalla (digital)?</v>
+      </c>
+      <c r="D23" t="str">
+        <v>fijo · digital</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="B24" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Cómo se comercializa. REGLA: si exhibicion=fijo solo "mensual" o "catorcenal".</v>
+      </c>
+      <c r="D24" t="str">
+        <v>mensual · catorcenal · semanal · diaria · spot · hora · programatico</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>es_rotativo</v>
+      </c>
+      <c r="B25" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C25" t="str">
+        <v>¿La cara rota entre varios anunciantes?</v>
+      </c>
+      <c r="D25" t="str">
+        <v>si · no</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>plaza_ciudad</v>
+      </c>
+      <c r="B26" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Ciudad o plaza donde está el sitio.</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>direccion</v>
+      </c>
+      <c r="B27" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Dirección o referencia de ubicación.</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>latitud</v>
+      </c>
+      <c r="B28" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Coordenada decimal. Si la dejas vacía, el sitio queda "pendiente de verificación".</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Número (ej. 19.4326)</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>longitud</v>
+      </c>
+      <c r="B29" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Coordenada decimal.</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Número (ej. -99.1332)</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>ancho_m</v>
+      </c>
+      <c r="B30" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Ancho de la pieza en metros.</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Número</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>alto_m</v>
+      </c>
+      <c r="B31" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Alto de la pieza en metros.</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Número</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>caras</v>
+      </c>
+      <c r="B32" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Número de caras del sitio (default 1).</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Número entero</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>iluminacion</v>
+      </c>
+      <c r="B33" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C33" t="str">
+        <v>¿Tiene iluminación?</v>
+      </c>
+      <c r="D33" t="str">
+        <v>si · no</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>tipo_estructura</v>
+      </c>
+      <c r="B34" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Tipo de estructura (unipolar, metálica, etc.).</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>vista</v>
+      </c>
+      <c r="B35" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Tipo de vista del tránsito.</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Texto libre (natural, cruzada…)</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>tramo</v>
+      </c>
+      <c r="B36" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Tramo o vialidad.</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>tarifa_publicada</v>
+      </c>
+      <c r="B37" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Precio de venta publicado (sin IVA), en la unidad indicada.</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Número</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>costo_compra</v>
+      </c>
+      <c r="B38" t="str">
+        <v>SÍ</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Tu costo de compra al proveedor (sin IVA).</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Número</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>spots_por_hora</v>
+      </c>
+      <c r="B39" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Solo DIGITAL: cuántos spots se reproducen por hora.</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Número (dejar vacío si es fijo)</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>duracion_spot_seg</v>
+      </c>
+      <c r="B40" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Solo DIGITAL: duración del spot en segundos.</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Número (dejar vacío si es fijo)</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>horario</v>
+      </c>
+      <c r="B41" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Horario de operación.</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Texto (ej. 06:00-23:00)</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>notas</v>
+      </c>
+      <c r="B42" t="str">
+        <v>opcional</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Notas adicionales.</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Texto libre</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D42"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:W3"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="19.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -470,9 +925,322 @@
         <v>notas</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>EJEMPLO-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Pantalla Periférico Sur</v>
+      </c>
+      <c r="C2" t="str">
+        <v>espectacular</v>
+      </c>
+      <c r="D2" t="str">
+        <v>digital</v>
+      </c>
+      <c r="E2" t="str">
+        <v>spot</v>
+      </c>
+      <c r="F2" t="str">
+        <v>no</v>
+      </c>
+      <c r="G2" t="str">
+        <v>CDMX</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Periférico Sur 4000</v>
+      </c>
+      <c r="I2">
+        <v>19.4326</v>
+      </c>
+      <c r="J2">
+        <v>-99.1332</v>
+      </c>
+      <c r="K2">
+        <v>12</v>
+      </c>
+      <c r="L2">
+        <v>7</v>
+      </c>
+      <c r="M2">
+        <v>1</v>
+      </c>
+      <c r="N2" t="str">
+        <v>si</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Estructura metálica</v>
+      </c>
+      <c r="P2" t="str">
+        <v>natural</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Periférico Sur</v>
+      </c>
+      <c r="R2">
+        <v>85000</v>
+      </c>
+      <c r="S2">
+        <v>52000</v>
+      </c>
+      <c r="T2">
+        <v>6</v>
+      </c>
+      <c r="U2">
+        <v>10</v>
+      </c>
+      <c r="V2" t="str">
+        <v>06:00-23:00</v>
+      </c>
+      <c r="W2" t="str">
+        <v>BORRA las filas EJEMPLO antes de importar</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>EJEMPLO-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Espectacular Insurgentes</v>
+      </c>
+      <c r="C3" t="str">
+        <v>espectacular</v>
+      </c>
+      <c r="D3" t="str">
+        <v>fijo</v>
+      </c>
+      <c r="E3" t="str">
+        <v>mensual</v>
+      </c>
+      <c r="F3" t="str">
+        <v>no</v>
+      </c>
+      <c r="G3" t="str">
+        <v>CDMX</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Av. Insurgentes 1200</v>
+      </c>
+      <c r="I3">
+        <v>19.39</v>
+      </c>
+      <c r="J3">
+        <v>-99.17</v>
+      </c>
+      <c r="K3">
+        <v>12</v>
+      </c>
+      <c r="L3">
+        <v>7</v>
+      </c>
+      <c r="M3">
+        <v>2</v>
+      </c>
+      <c r="N3" t="str">
+        <v>si</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Unipolar</v>
+      </c>
+      <c r="P3" t="str">
+        <v>cruzada</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Insurgentes Sur</v>
+      </c>
+      <c r="R3">
+        <v>45000</v>
+      </c>
+      <c r="S3">
+        <v>28000</v>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v>BORRA las filas EJEMPLO antes de importar</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E9"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="8.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>exhibicion</v>
+      </c>
+      <c r="B1" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="C1" t="str">
+        <v>unidad_si_es_fijo</v>
+      </c>
+      <c r="D1" t="str">
+        <v>tipo_medio</v>
+      </c>
+      <c r="E1" t="str">
+        <v>si_no</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>fijo</v>
+      </c>
+      <c r="B2" t="str">
+        <v>mensual</v>
+      </c>
+      <c r="C2" t="str">
+        <v>mensual</v>
+      </c>
+      <c r="D2" t="str">
+        <v>espectacular</v>
+      </c>
+      <c r="E2" t="str">
+        <v>si</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>digital</v>
+      </c>
+      <c r="B3" t="str">
+        <v>catorcenal</v>
+      </c>
+      <c r="C3" t="str">
+        <v>catorcenal</v>
+      </c>
+      <c r="D3" t="str">
+        <v>muro</v>
+      </c>
+      <c r="E3" t="str">
+        <v>no</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v>semanal</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>valla</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v>diaria</v>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>parabus</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v>spot</v>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>mupi</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v>hora</v>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>publitienda</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v>programatico</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>puente</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>otro</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>